<commit_message>
correzione excel con rates a frazione
</commit_message>
<xml_diff>
--- a/Pipe_Matlab_Indici_di_Prestazione_Guasto/FOLDER/EXCEL.xlsx
+++ b/Pipe_Matlab_Indici_di_Prestazione_Guasto/FOLDER/EXCEL.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lachiara\Desktop\Uni_Andrea\Magistrale\Secondo_Anno\Controllo_Avanzato\Pipe_Matlab\FOLDER\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lachiara\Documents\GitHub\ControlloAvanzato\Pipe_Matlab_Indici_di_Prestazione_Guasto\FOLDER\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08ACB2A3-2FAB-45C9-9941-667B68F1F74D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{903102EF-238B-47B3-AADA-BAC616E5287F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="67">
   <si>
     <t>Petri net incidence and marking</t>
   </si>
@@ -289,21 +289,6 @@
     <t>rates</t>
   </si>
   <si>
-    <t xml:space="preserve"> 1/2</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1/6</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1/5</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1/8</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1/3</t>
-  </si>
-  <si>
     <t>pesi</t>
   </si>
   <si>
@@ -311,6 +296,12 @@
   </si>
   <si>
     <t>servers</t>
+  </si>
+  <si>
+    <t>5 minuti</t>
+  </si>
+  <si>
+    <t>2 minuti</t>
   </si>
 </sst>
 </file>
@@ -396,7 +387,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -421,6 +412,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -434,7 +431,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -454,13 +451,16 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="12" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="12" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -741,7 +741,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AE150"/>
+  <dimension ref="A1:AE153"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="19" max="19" width="9.21875" bestFit="1" customWidth="1"/>
@@ -753,28 +753,28 @@
       </c>
     </row>
     <row r="3" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
-      <c r="L3" s="7"/>
-      <c r="M3" s="7"/>
-      <c r="N3" s="7"/>
-      <c r="O3" s="7"/>
-      <c r="P3" s="7"/>
-      <c r="Q3" s="7"/>
-      <c r="R3" s="7"/>
-      <c r="S3" s="7"/>
-      <c r="T3" s="7"/>
+      <c r="A3" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="8"/>
+      <c r="O3" s="8"/>
+      <c r="P3" s="8"/>
+      <c r="Q3" s="8"/>
+      <c r="R3" s="8"/>
+      <c r="S3" s="8"/>
+      <c r="T3" s="8"/>
     </row>
     <row r="4" spans="1:20" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
@@ -2697,28 +2697,28 @@
       </c>
     </row>
     <row r="35" spans="1:20" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="8" t="s">
+      <c r="A35" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B35" s="8"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="8"/>
-      <c r="E35" s="8"/>
-      <c r="F35" s="8"/>
-      <c r="G35" s="8"/>
-      <c r="H35" s="8"/>
-      <c r="I35" s="8"/>
-      <c r="J35" s="8"/>
-      <c r="K35" s="8"/>
-      <c r="L35" s="8"/>
-      <c r="M35" s="8"/>
-      <c r="N35" s="8"/>
-      <c r="O35" s="8"/>
-      <c r="P35" s="8"/>
-      <c r="Q35" s="8"/>
-      <c r="R35" s="8"/>
-      <c r="S35" s="8"/>
-      <c r="T35" s="8"/>
+      <c r="B35" s="7"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="7"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="7"/>
+      <c r="G35" s="7"/>
+      <c r="H35" s="7"/>
+      <c r="I35" s="7"/>
+      <c r="J35" s="7"/>
+      <c r="K35" s="7"/>
+      <c r="L35" s="7"/>
+      <c r="M35" s="7"/>
+      <c r="N35" s="7"/>
+      <c r="O35" s="7"/>
+      <c r="P35" s="7"/>
+      <c r="Q35" s="7"/>
+      <c r="R35" s="7"/>
+      <c r="S35" s="7"/>
+      <c r="T35" s="7"/>
     </row>
     <row r="36" spans="1:20" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A36" s="2"/>
@@ -4641,28 +4641,28 @@
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A67" s="8" t="s">
+      <c r="A67" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B67" s="8"/>
-      <c r="C67" s="8"/>
-      <c r="D67" s="8"/>
-      <c r="E67" s="8"/>
-      <c r="F67" s="8"/>
-      <c r="G67" s="8"/>
-      <c r="H67" s="8"/>
-      <c r="I67" s="8"/>
-      <c r="J67" s="8"/>
-      <c r="K67" s="8"/>
-      <c r="L67" s="8"/>
-      <c r="M67" s="8"/>
-      <c r="N67" s="8"/>
-      <c r="O67" s="8"/>
-      <c r="P67" s="8"/>
-      <c r="Q67" s="8"/>
-      <c r="R67" s="8"/>
-      <c r="S67" s="8"/>
-      <c r="T67" s="8"/>
+      <c r="B67" s="7"/>
+      <c r="C67" s="7"/>
+      <c r="D67" s="7"/>
+      <c r="E67" s="7"/>
+      <c r="F67" s="7"/>
+      <c r="G67" s="7"/>
+      <c r="H67" s="7"/>
+      <c r="I67" s="7"/>
+      <c r="J67" s="7"/>
+      <c r="K67" s="7"/>
+      <c r="L67" s="7"/>
+      <c r="M67" s="7"/>
+      <c r="N67" s="7"/>
+      <c r="O67" s="7"/>
+      <c r="P67" s="7"/>
+      <c r="Q67" s="7"/>
+      <c r="R67" s="7"/>
+      <c r="S67" s="7"/>
+      <c r="T67" s="7"/>
     </row>
     <row r="68" spans="1:20" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A68" s="2"/>
@@ -6585,28 +6585,28 @@
       </c>
     </row>
     <row r="99" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A99" s="8" t="s">
+      <c r="A99" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B99" s="8"/>
-      <c r="C99" s="8"/>
-      <c r="D99" s="8"/>
-      <c r="E99" s="8"/>
-      <c r="F99" s="8"/>
-      <c r="G99" s="8"/>
-      <c r="H99" s="8"/>
-      <c r="I99" s="8"/>
-      <c r="J99" s="8"/>
-      <c r="K99" s="8"/>
-      <c r="L99" s="8"/>
-      <c r="M99" s="8"/>
-      <c r="N99" s="8"/>
-      <c r="O99" s="8"/>
-      <c r="P99" s="8"/>
-      <c r="Q99" s="8"/>
-      <c r="R99" s="8"/>
-      <c r="S99" s="8"/>
-      <c r="T99" s="8"/>
+      <c r="B99" s="7"/>
+      <c r="C99" s="7"/>
+      <c r="D99" s="7"/>
+      <c r="E99" s="7"/>
+      <c r="F99" s="7"/>
+      <c r="G99" s="7"/>
+      <c r="H99" s="7"/>
+      <c r="I99" s="7"/>
+      <c r="J99" s="7"/>
+      <c r="K99" s="7"/>
+      <c r="L99" s="7"/>
+      <c r="M99" s="7"/>
+      <c r="N99" s="7"/>
+      <c r="O99" s="7"/>
+      <c r="P99" s="7"/>
+      <c r="Q99" s="7"/>
+      <c r="R99" s="7"/>
+      <c r="S99" s="7"/>
+      <c r="T99" s="7"/>
     </row>
     <row r="100" spans="1:20" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A100" s="2"/>
@@ -8529,39 +8529,39 @@
       </c>
     </row>
     <row r="131" spans="1:31" x14ac:dyDescent="0.3">
-      <c r="A131" s="8" t="s">
+      <c r="A131" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="B131" s="8"/>
-      <c r="C131" s="8"/>
-      <c r="D131" s="8"/>
-      <c r="E131" s="8"/>
-      <c r="F131" s="8"/>
-      <c r="G131" s="8"/>
-      <c r="H131" s="8"/>
-      <c r="I131" s="8"/>
-      <c r="J131" s="8"/>
-      <c r="K131" s="8"/>
-      <c r="L131" s="8"/>
-      <c r="M131" s="8"/>
-      <c r="N131" s="8"/>
-      <c r="O131" s="8"/>
-      <c r="P131" s="8"/>
-      <c r="Q131" s="8"/>
-      <c r="R131" s="8"/>
-      <c r="S131" s="8"/>
-      <c r="T131" s="8"/>
-      <c r="U131" s="8"/>
-      <c r="V131" s="8"/>
-      <c r="W131" s="8"/>
-      <c r="X131" s="8"/>
-      <c r="Y131" s="8"/>
-      <c r="Z131" s="8"/>
-      <c r="AA131" s="8"/>
-      <c r="AB131" s="8"/>
-      <c r="AC131" s="8"/>
-      <c r="AD131" s="8"/>
-      <c r="AE131" s="8"/>
+      <c r="B131" s="7"/>
+      <c r="C131" s="7"/>
+      <c r="D131" s="7"/>
+      <c r="E131" s="7"/>
+      <c r="F131" s="7"/>
+      <c r="G131" s="7"/>
+      <c r="H131" s="7"/>
+      <c r="I131" s="7"/>
+      <c r="J131" s="7"/>
+      <c r="K131" s="7"/>
+      <c r="L131" s="7"/>
+      <c r="M131" s="7"/>
+      <c r="N131" s="7"/>
+      <c r="O131" s="7"/>
+      <c r="P131" s="7"/>
+      <c r="Q131" s="7"/>
+      <c r="R131" s="7"/>
+      <c r="S131" s="7"/>
+      <c r="T131" s="7"/>
+      <c r="U131" s="7"/>
+      <c r="V131" s="7"/>
+      <c r="W131" s="7"/>
+      <c r="X131" s="7"/>
+      <c r="Y131" s="7"/>
+      <c r="Z131" s="7"/>
+      <c r="AA131" s="7"/>
+      <c r="AB131" s="7"/>
+      <c r="AC131" s="7"/>
+      <c r="AD131" s="7"/>
+      <c r="AE131" s="7"/>
     </row>
     <row r="132" spans="1:31" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A132" s="2"/>
@@ -8847,27 +8847,27 @@
       </c>
     </row>
     <row r="135" spans="1:31" x14ac:dyDescent="0.3">
-      <c r="A135" s="8" t="s">
+      <c r="A135" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B135" s="8"/>
-      <c r="C135" s="8"/>
-      <c r="D135" s="8"/>
-      <c r="E135" s="8"/>
-      <c r="F135" s="8"/>
-      <c r="G135" s="8"/>
-      <c r="H135" s="8"/>
-      <c r="I135" s="8"/>
-      <c r="J135" s="8"/>
-      <c r="K135" s="8"/>
-      <c r="L135" s="8"/>
-      <c r="M135" s="8"/>
-      <c r="N135" s="8"/>
-      <c r="O135" s="8"/>
-      <c r="P135" s="8"/>
-      <c r="Q135" s="8"/>
-      <c r="R135" s="8"/>
-      <c r="S135" s="8"/>
+      <c r="B135" s="7"/>
+      <c r="C135" s="7"/>
+      <c r="D135" s="7"/>
+      <c r="E135" s="7"/>
+      <c r="F135" s="7"/>
+      <c r="G135" s="7"/>
+      <c r="H135" s="7"/>
+      <c r="I135" s="7"/>
+      <c r="J135" s="7"/>
+      <c r="K135" s="7"/>
+      <c r="L135" s="7"/>
+      <c r="M135" s="7"/>
+      <c r="N135" s="7"/>
+      <c r="O135" s="7"/>
+      <c r="P135" s="7"/>
+      <c r="Q135" s="7"/>
+      <c r="R135" s="7"/>
+      <c r="S135" s="7"/>
     </row>
     <row r="136" spans="1:31" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A136" s="3" t="s">
@@ -9180,56 +9180,56 @@
       </c>
     </row>
     <row r="144" spans="1:31" x14ac:dyDescent="0.3">
-      <c r="A144" t="s">
-        <v>62</v>
-      </c>
-      <c r="B144" t="s">
-        <v>63</v>
-      </c>
-      <c r="C144" t="s">
-        <v>62</v>
-      </c>
-      <c r="D144">
-        <v>0</v>
-      </c>
-      <c r="E144">
-        <v>0</v>
-      </c>
-      <c r="F144">
-        <v>0</v>
-      </c>
-      <c r="G144">
-        <v>0</v>
-      </c>
-      <c r="H144" t="s">
-        <v>62</v>
-      </c>
-      <c r="I144" t="s">
-        <v>64</v>
-      </c>
-      <c r="J144" t="s">
-        <v>62</v>
-      </c>
-      <c r="K144">
-        <v>0</v>
-      </c>
-      <c r="L144" t="s">
-        <v>62</v>
-      </c>
-      <c r="M144" t="s">
-        <v>64</v>
-      </c>
-      <c r="N144" t="s">
-        <v>62</v>
-      </c>
-      <c r="O144">
-        <v>0</v>
-      </c>
-      <c r="P144" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q144" t="s">
-        <v>66</v>
+      <c r="A144" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="B144" s="9">
+        <v>0.16</v>
+      </c>
+      <c r="C144" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="D144" s="9">
+        <v>0</v>
+      </c>
+      <c r="E144" s="9">
+        <v>0</v>
+      </c>
+      <c r="F144" s="9">
+        <v>0</v>
+      </c>
+      <c r="G144" s="9">
+        <v>0</v>
+      </c>
+      <c r="H144" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="I144" s="9">
+        <v>0.2</v>
+      </c>
+      <c r="J144" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="K144" s="9">
+        <v>0</v>
+      </c>
+      <c r="L144" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="M144" s="9">
+        <v>0.2</v>
+      </c>
+      <c r="N144" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="O144" s="9">
+        <v>0</v>
+      </c>
+      <c r="P144" s="9">
+        <v>0.125</v>
+      </c>
+      <c r="Q144" s="9">
+        <v>0.33</v>
       </c>
       <c r="R144" s="9">
         <v>0.2</v>
@@ -9240,7 +9240,7 @@
     </row>
     <row r="145" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="146" spans="1:19" x14ac:dyDescent="0.3">
@@ -9304,7 +9304,7 @@
     </row>
     <row r="147" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
     <row r="148" spans="1:19" x14ac:dyDescent="0.3">
@@ -9368,7 +9368,7 @@
     </row>
     <row r="149" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
     <row r="150" spans="1:19" x14ac:dyDescent="0.3">
@@ -9428,6 +9428,14 @@
       </c>
       <c r="S150">
         <v>0</v>
+      </c>
+    </row>
+    <row r="153" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="R153" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="S153" s="10" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
correzione rete con guasto
</commit_message>
<xml_diff>
--- a/Pipe_Matlab_Indici_di_Prestazione_Guasto/FOLDER/EXCEL.xlsx
+++ b/Pipe_Matlab_Indici_di_Prestazione_Guasto/FOLDER/EXCEL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lachiara\Documents\GitHub\ControlloAvanzato\Pipe_Matlab_Indici_di_Prestazione_Guasto\FOLDER\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8001189D-AEEE-4597-8189-E62A66E3EED4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CD21B90-0B80-4BEC-A069-51EAA88DEB79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="65">
   <si>
     <t>Petri net incidence and marking</t>
   </si>
@@ -70,6 +70,12 @@
     <t>Ant_Post_Scarico_Buffer</t>
   </si>
   <si>
+    <t>Ant_Post_Tagliatrice_Pressa_Guasto</t>
+  </si>
+  <si>
+    <t>Ant_Post_Tagliatrice_Pressa_Riparata</t>
+  </si>
+  <si>
     <t>Carico_Laminati</t>
   </si>
   <si>
@@ -109,12 +115,6 @@
     <t>Trasporto_Laminati</t>
   </si>
   <si>
-    <t>Ant_Post_Tagliatrice_Pressa_Riparata</t>
-  </si>
-  <si>
-    <t>Ant_Post_Tagliatrice_Pressa_Guasto</t>
-  </si>
-  <si>
     <t>Ant_Post_Conforme</t>
   </si>
   <si>
@@ -124,16 +124,22 @@
     <t>Ant_Post_Disp_Conforme</t>
   </si>
   <si>
-    <t>Ant_Post_Grezzi_Tagl_Press</t>
+    <t>Ant_Post_Grezzo</t>
+  </si>
+  <si>
+    <t>Ant_Post_Lavorato</t>
   </si>
   <si>
     <t>Ant_Post_Pezzi_Buffer</t>
   </si>
   <si>
-    <t>Ant_Post_Tagliato_Pressato</t>
+    <t>Ant_Post_Tagl_Press</t>
   </si>
   <si>
     <t>Ant_Post_Tagliatrice_Pressa</t>
+  </si>
+  <si>
+    <t>Ant_Post_Tagliatrice_Pressa_Guasta</t>
   </si>
   <si>
     <t>Carrozzeria_Pronta</t>
@@ -160,16 +166,16 @@
     <t>Lat_Dx_Disp_Conforme</t>
   </si>
   <si>
-    <t>Lat_Dx_Grezzi_Tagl_Press</t>
+    <t>Lat_Dx_Grezzo</t>
   </si>
   <si>
-    <t>Lat_Dx_Grezzo</t>
+    <t>Lat_Dx_Lavorato</t>
   </si>
   <si>
     <t>Lat_Dx_Pezzi_Buffer</t>
   </si>
   <si>
-    <t>Lat_Dx_Tagliato_Pressato</t>
+    <t>Lat_Dx_Tagl_Press</t>
   </si>
   <si>
     <t>Lat_Dx_Tagliatrice_Pressa</t>
@@ -184,25 +190,19 @@
     <t>Lat_Sx_Disp_Conforme</t>
   </si>
   <si>
-    <t>Lat_Sx_Greezzi_Tagl_Press</t>
+    <t>Lat_Sx_Grezzo</t>
   </si>
   <si>
-    <t>Lat_Sx_Grezzo</t>
+    <t>Lat_Sx_Lavorato</t>
   </si>
   <si>
     <t>Lat_Sx_Pezzi_Buffer</t>
   </si>
   <si>
-    <t>Lat_Sx_Tagliato_Pressato</t>
+    <t>Lat_Sx_Tagl_Press</t>
   </si>
   <si>
     <t>Lat_Sx_Tagliatrice_Pressa</t>
-  </si>
-  <si>
-    <t>Pezzo_Ant_Post_sul_Nastro</t>
-  </si>
-  <si>
-    <t>Ant_Post_Tagliatrice_Pressa_Guasta</t>
   </si>
   <si>
     <r>
@@ -297,12 +297,6 @@
   <si>
     <t>servers</t>
   </si>
-  <si>
-    <t>5 minuti</t>
-  </si>
-  <si>
-    <t>2 minuti</t>
-  </si>
 </sst>
 </file>
 
@@ -387,7 +381,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -412,12 +406,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -431,7 +419,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -451,15 +439,14 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="12" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="12" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -741,11 +728,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AE153"/>
+  <dimension ref="A1:AE150"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="19" max="19" width="9.21875" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -753,28 +737,28 @@
       </c>
     </row>
     <row r="3" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="10"/>
-      <c r="Q3" s="10"/>
-      <c r="R3" s="10"/>
-      <c r="S3" s="10"/>
-      <c r="T3" s="10"/>
+      <c r="A3" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="7"/>
+      <c r="T3" s="7"/>
     </row>
     <row r="4" spans="1:20" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
@@ -1010,24 +994,24 @@
         <v>0</v>
       </c>
       <c r="Q7" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R7" s="5">
         <v>0</v>
       </c>
       <c r="S7" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T7" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>24</v>
       </c>
       <c r="B8" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C8" s="6">
         <v>0</v>
@@ -1048,7 +1032,7 @@
         <v>0</v>
       </c>
       <c r="I8" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8" s="6">
         <v>0</v>
@@ -1084,7 +1068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>25</v>
       </c>
@@ -1092,10 +1076,10 @@
         <v>0</v>
       </c>
       <c r="C9" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" s="5">
         <v>0</v>
@@ -1154,10 +1138,10 @@
         <v>0</v>
       </c>
       <c r="C10" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D10" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" s="6">
         <v>0</v>
@@ -1213,13 +1197,13 @@
         <v>27</v>
       </c>
       <c r="B11" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C11" s="5">
         <v>0</v>
       </c>
       <c r="D11" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11" s="5">
         <v>0</v>
@@ -1264,13 +1248,13 @@
         <v>0</v>
       </c>
       <c r="S11" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T11" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>28</v>
       </c>
@@ -1281,7 +1265,7 @@
         <v>0</v>
       </c>
       <c r="D12" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" s="6">
         <v>0</v>
@@ -1290,7 +1274,7 @@
         <v>0</v>
       </c>
       <c r="G12" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12" s="6">
         <v>0</v>
@@ -1320,7 +1304,7 @@
         <v>0</v>
       </c>
       <c r="Q12" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R12" s="6">
         <v>0</v>
@@ -1332,7 +1316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:20" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>29</v>
       </c>
@@ -1349,10 +1333,10 @@
         <v>0</v>
       </c>
       <c r="F13" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H13" s="5">
         <v>0</v>
@@ -1394,7 +1378,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>30</v>
       </c>
@@ -1411,7 +1395,7 @@
         <v>0</v>
       </c>
       <c r="F14" s="6">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G14" s="6">
         <v>0</v>
@@ -1450,13 +1434,13 @@
         <v>0</v>
       </c>
       <c r="S14" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T14" s="6">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>31</v>
       </c>
@@ -1482,7 +1466,7 @@
         <v>0</v>
       </c>
       <c r="I15" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J15" s="5">
         <v>0</v>
@@ -1509,7 +1493,7 @@
         <v>0</v>
       </c>
       <c r="R15" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S15" s="5">
         <v>0</v>
@@ -1518,7 +1502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>32</v>
       </c>
@@ -1541,7 +1525,7 @@
         <v>0</v>
       </c>
       <c r="H16" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I16" s="6">
         <v>0</v>
@@ -1580,7 +1564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>33</v>
       </c>
@@ -1615,7 +1599,7 @@
         <v>0</v>
       </c>
       <c r="L17" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M17" s="5">
         <v>0</v>
@@ -1639,10 +1623,10 @@
         <v>0</v>
       </c>
       <c r="T17" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>34</v>
       </c>
@@ -1671,13 +1655,13 @@
         <v>0</v>
       </c>
       <c r="J18" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18" s="6">
         <v>0</v>
       </c>
       <c r="L18" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M18" s="6">
         <v>0</v>
@@ -1704,7 +1688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>35</v>
       </c>
@@ -1745,7 +1729,7 @@
         <v>0</v>
       </c>
       <c r="N19" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O19" s="5">
         <v>0</v>
@@ -1754,7 +1738,7 @@
         <v>0</v>
       </c>
       <c r="Q19" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R19" s="5">
         <v>0</v>
@@ -1766,7 +1750,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>36</v>
       </c>
@@ -1792,7 +1776,7 @@
         <v>0</v>
       </c>
       <c r="I20" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20" s="6">
         <v>0</v>
@@ -1807,7 +1791,7 @@
         <v>0</v>
       </c>
       <c r="N20" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O20" s="6">
         <v>0</v>
@@ -1828,7 +1812,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>37</v>
       </c>
@@ -1848,7 +1832,7 @@
         <v>0</v>
       </c>
       <c r="G21" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H21" s="5">
         <v>0</v>
@@ -1884,13 +1868,13 @@
         <v>0</v>
       </c>
       <c r="S21" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T21" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>38</v>
       </c>
@@ -1916,13 +1900,13 @@
         <v>0</v>
       </c>
       <c r="I22" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" s="6">
         <v>0</v>
       </c>
       <c r="K22" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L22" s="6">
         <v>0</v>
@@ -1952,7 +1936,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>39</v>
       </c>
@@ -1981,13 +1965,13 @@
         <v>0</v>
       </c>
       <c r="J23" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K23" s="5">
         <v>0</v>
       </c>
       <c r="L23" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M23" s="5">
         <v>0</v>
@@ -2046,13 +2030,13 @@
         <v>0</v>
       </c>
       <c r="K24" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L24" s="6">
         <v>0</v>
       </c>
       <c r="M24" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N24" s="6">
         <v>0</v>
@@ -2108,7 +2092,7 @@
         <v>0</v>
       </c>
       <c r="K25" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L25" s="5">
         <v>0</v>
@@ -2123,7 +2107,7 @@
         <v>0</v>
       </c>
       <c r="P25" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q25" s="5">
         <v>0</v>
@@ -2138,7 +2122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>42</v>
       </c>
@@ -2176,7 +2160,7 @@
         <v>0</v>
       </c>
       <c r="M26" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N26" s="6">
         <v>0</v>
@@ -2185,7 +2169,7 @@
         <v>0</v>
       </c>
       <c r="P26" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q26" s="6">
         <v>0</v>
@@ -2200,7 +2184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>43</v>
       </c>
@@ -2250,10 +2234,10 @@
         <v>0</v>
       </c>
       <c r="Q27" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R27" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S27" s="5">
         <v>0</v>
@@ -2262,7 +2246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>44</v>
       </c>
@@ -2300,7 +2284,7 @@
         <v>0</v>
       </c>
       <c r="M28" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N28" s="6">
         <v>0</v>
@@ -2315,7 +2299,7 @@
         <v>0</v>
       </c>
       <c r="R28" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S28" s="6">
         <v>0</v>
@@ -2324,7 +2308,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>45</v>
       </c>
@@ -2344,7 +2328,7 @@
         <v>0</v>
       </c>
       <c r="G29" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H29" s="5">
         <v>0</v>
@@ -2380,7 +2364,7 @@
         <v>0</v>
       </c>
       <c r="S29" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T29" s="5">
         <v>0</v>
@@ -2412,7 +2396,7 @@
         <v>0</v>
       </c>
       <c r="I30" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J30" s="6">
         <v>0</v>
@@ -2430,7 +2414,7 @@
         <v>0</v>
       </c>
       <c r="O30" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P30" s="6">
         <v>0</v>
@@ -2448,7 +2432,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>47</v>
       </c>
@@ -2489,13 +2473,13 @@
         <v>0</v>
       </c>
       <c r="N31" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O31" s="5">
         <v>0</v>
       </c>
       <c r="P31" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q31" s="5">
         <v>0</v>
@@ -2510,7 +2494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>48</v>
       </c>
@@ -2554,13 +2538,13 @@
         <v>0</v>
       </c>
       <c r="O32" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P32" s="6">
         <v>0</v>
       </c>
       <c r="Q32" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R32" s="6">
         <v>0</v>
@@ -2572,7 +2556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>49</v>
       </c>
@@ -2592,7 +2576,7 @@
         <v>0</v>
       </c>
       <c r="G33" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H33" s="5">
         <v>0</v>
@@ -2616,7 +2600,7 @@
         <v>0</v>
       </c>
       <c r="O33" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P33" s="5">
         <v>0</v>
@@ -2634,7 +2618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:20" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>50</v>
       </c>
@@ -2684,7 +2668,7 @@
         <v>0</v>
       </c>
       <c r="Q34" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R34" s="6">
         <v>0</v>
@@ -2693,32 +2677,32 @@
         <v>0</v>
       </c>
       <c r="T34" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:20" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="9" t="s">
+      <c r="A35" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B35" s="9"/>
-      <c r="C35" s="9"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="9"/>
-      <c r="G35" s="9"/>
-      <c r="H35" s="9"/>
-      <c r="I35" s="9"/>
-      <c r="J35" s="9"/>
-      <c r="K35" s="9"/>
-      <c r="L35" s="9"/>
-      <c r="M35" s="9"/>
-      <c r="N35" s="9"/>
-      <c r="O35" s="9"/>
-      <c r="P35" s="9"/>
-      <c r="Q35" s="9"/>
-      <c r="R35" s="9"/>
-      <c r="S35" s="9"/>
-      <c r="T35" s="9"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="8"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="8"/>
+      <c r="I35" s="8"/>
+      <c r="J35" s="8"/>
+      <c r="K35" s="8"/>
+      <c r="L35" s="8"/>
+      <c r="M35" s="8"/>
+      <c r="N35" s="8"/>
+      <c r="O35" s="8"/>
+      <c r="P35" s="8"/>
+      <c r="Q35" s="8"/>
+      <c r="R35" s="8"/>
+      <c r="S35" s="8"/>
+      <c r="T35" s="8"/>
     </row>
     <row r="36" spans="1:20" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A36" s="2"/>
@@ -2830,13 +2814,13 @@
         <v>0</v>
       </c>
       <c r="Q37" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R37" s="5">
         <v>0</v>
       </c>
       <c r="S37" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T37" s="5">
         <v>0</v>
@@ -2966,15 +2950,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
         <v>24</v>
       </c>
       <c r="B40" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C40" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D40" s="6">
         <v>0</v>
@@ -3028,7 +3012,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
         <v>25</v>
       </c>
@@ -3039,10 +3023,10 @@
         <v>0</v>
       </c>
       <c r="D41" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E41" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F41" s="5">
         <v>0</v>
@@ -3101,10 +3085,10 @@
         <v>0</v>
       </c>
       <c r="D42" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E42" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F42" s="6">
         <v>0</v>
@@ -3157,10 +3141,10 @@
         <v>27</v>
       </c>
       <c r="B43" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C43" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D43" s="5">
         <v>0</v>
@@ -3211,15 +3195,15 @@
         <v>0</v>
       </c>
       <c r="T43" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>28</v>
       </c>
       <c r="B44" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C44" s="6">
         <v>0</v>
@@ -3276,7 +3260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:20" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
         <v>29</v>
       </c>
@@ -3296,10 +3280,10 @@
         <v>0</v>
       </c>
       <c r="G45" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H45" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I45" s="5">
         <v>0</v>
@@ -3338,7 +3322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
         <v>30</v>
       </c>
@@ -3361,7 +3345,7 @@
         <v>0</v>
       </c>
       <c r="H46" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I46" s="6">
         <v>0</v>
@@ -3400,7 +3384,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
         <v>31</v>
       </c>
@@ -3420,7 +3404,7 @@
         <v>0</v>
       </c>
       <c r="G47" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H47" s="5">
         <v>0</v>
@@ -3429,7 +3413,7 @@
         <v>0</v>
       </c>
       <c r="J47" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K47" s="5">
         <v>0</v>
@@ -3462,7 +3446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
         <v>32</v>
       </c>
@@ -3491,7 +3475,7 @@
         <v>0</v>
       </c>
       <c r="J48" s="6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K48" s="6">
         <v>0</v>
@@ -3515,7 +3499,7 @@
         <v>0</v>
       </c>
       <c r="R48" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S48" s="6">
         <v>0</v>
@@ -3524,7 +3508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A49" s="4" t="s">
         <v>33</v>
       </c>
@@ -3550,7 +3534,7 @@
         <v>0</v>
       </c>
       <c r="I49" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J49" s="5">
         <v>0</v>
@@ -3574,7 +3558,7 @@
         <v>0</v>
       </c>
       <c r="Q49" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R49" s="5">
         <v>0</v>
@@ -3586,7 +3570,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
         <v>34</v>
       </c>
@@ -3618,7 +3602,7 @@
         <v>0</v>
       </c>
       <c r="K50" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L50" s="6">
         <v>0</v>
@@ -3645,10 +3629,10 @@
         <v>0</v>
       </c>
       <c r="T50" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A51" s="4" t="s">
         <v>35</v>
       </c>
@@ -3683,7 +3667,7 @@
         <v>0</v>
       </c>
       <c r="L51" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M51" s="5">
         <v>0</v>
@@ -3704,13 +3688,13 @@
         <v>0</v>
       </c>
       <c r="S51" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T51" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
         <v>36</v>
       </c>
@@ -3739,7 +3723,7 @@
         <v>0</v>
       </c>
       <c r="J52" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K52" s="6">
         <v>0</v>
@@ -3748,7 +3732,7 @@
         <v>0</v>
       </c>
       <c r="M52" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N52" s="6">
         <v>0</v>
@@ -3772,7 +3756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A53" s="4" t="s">
         <v>37</v>
       </c>
@@ -3798,7 +3782,7 @@
         <v>0</v>
       </c>
       <c r="I53" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J53" s="5">
         <v>0</v>
@@ -3813,7 +3797,7 @@
         <v>0</v>
       </c>
       <c r="N53" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O53" s="5">
         <v>0</v>
@@ -3834,7 +3818,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
         <v>38</v>
       </c>
@@ -3866,10 +3850,10 @@
         <v>0</v>
       </c>
       <c r="K54" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L54" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M54" s="6">
         <v>0</v>
@@ -3896,7 +3880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A55" s="4" t="s">
         <v>39</v>
       </c>
@@ -3928,13 +3912,13 @@
         <v>0</v>
       </c>
       <c r="K55" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L55" s="5">
         <v>0</v>
       </c>
       <c r="M55" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N55" s="5">
         <v>0</v>
@@ -3984,7 +3968,7 @@
         <v>0</v>
       </c>
       <c r="I56" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J56" s="6">
         <v>0</v>
@@ -3999,7 +3983,7 @@
         <v>0</v>
       </c>
       <c r="N56" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O56" s="6">
         <v>0</v>
@@ -4055,7 +4039,7 @@
         <v>0</v>
       </c>
       <c r="L57" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M57" s="5">
         <v>0</v>
@@ -4070,7 +4054,7 @@
         <v>0</v>
       </c>
       <c r="Q57" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R57" s="5">
         <v>0</v>
@@ -4082,7 +4066,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
         <v>42</v>
       </c>
@@ -4114,7 +4098,7 @@
         <v>0</v>
       </c>
       <c r="K58" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L58" s="6">
         <v>0</v>
@@ -4126,7 +4110,7 @@
         <v>0</v>
       </c>
       <c r="O58" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P58" s="6">
         <v>0</v>
@@ -4144,7 +4128,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
         <v>43</v>
       </c>
@@ -4191,7 +4175,7 @@
         <v>0</v>
       </c>
       <c r="P59" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q59" s="5">
         <v>0</v>
@@ -4200,13 +4184,13 @@
         <v>0</v>
       </c>
       <c r="S59" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T59" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
         <v>44</v>
       </c>
@@ -4247,7 +4231,7 @@
         <v>0</v>
       </c>
       <c r="N60" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O60" s="6">
         <v>0</v>
@@ -4256,7 +4240,7 @@
         <v>0</v>
       </c>
       <c r="Q60" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R60" s="6">
         <v>0</v>
@@ -4268,7 +4252,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
         <v>45</v>
       </c>
@@ -4306,7 +4290,7 @@
         <v>0</v>
       </c>
       <c r="M61" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N61" s="5">
         <v>0</v>
@@ -4321,7 +4305,7 @@
         <v>0</v>
       </c>
       <c r="R61" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S61" s="5">
         <v>0</v>
@@ -4374,10 +4358,10 @@
         <v>0</v>
       </c>
       <c r="O62" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P62" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q62" s="6">
         <v>0</v>
@@ -4392,7 +4376,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
         <v>47</v>
       </c>
@@ -4436,13 +4420,13 @@
         <v>0</v>
       </c>
       <c r="O63" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P63" s="5">
         <v>0</v>
       </c>
       <c r="Q63" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R63" s="5">
         <v>0</v>
@@ -4454,7 +4438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
         <v>48</v>
       </c>
@@ -4492,7 +4476,7 @@
         <v>0</v>
       </c>
       <c r="M64" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N64" s="6">
         <v>0</v>
@@ -4507,7 +4491,7 @@
         <v>0</v>
       </c>
       <c r="R64" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S64" s="6">
         <v>0</v>
@@ -4516,12 +4500,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A65" s="4" t="s">
         <v>49</v>
       </c>
       <c r="B65" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C65" s="5">
         <v>0</v>
@@ -4563,7 +4547,7 @@
         <v>0</v>
       </c>
       <c r="P65" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q65" s="5">
         <v>0</v>
@@ -4578,7 +4562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:20" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
         <v>50</v>
       </c>
@@ -4622,7 +4606,7 @@
         <v>0</v>
       </c>
       <c r="O66" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P66" s="6">
         <v>0</v>
@@ -4634,35 +4618,35 @@
         <v>0</v>
       </c>
       <c r="S66" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T66" s="6">
         <v>0</v>
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A67" s="9" t="s">
+      <c r="A67" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B67" s="9"/>
-      <c r="C67" s="9"/>
-      <c r="D67" s="9"/>
-      <c r="E67" s="9"/>
-      <c r="F67" s="9"/>
-      <c r="G67" s="9"/>
-      <c r="H67" s="9"/>
-      <c r="I67" s="9"/>
-      <c r="J67" s="9"/>
-      <c r="K67" s="9"/>
-      <c r="L67" s="9"/>
-      <c r="M67" s="9"/>
-      <c r="N67" s="9"/>
-      <c r="O67" s="9"/>
-      <c r="P67" s="9"/>
-      <c r="Q67" s="9"/>
-      <c r="R67" s="9"/>
-      <c r="S67" s="9"/>
-      <c r="T67" s="9"/>
+      <c r="B67" s="8"/>
+      <c r="C67" s="8"/>
+      <c r="D67" s="8"/>
+      <c r="E67" s="8"/>
+      <c r="F67" s="8"/>
+      <c r="G67" s="8"/>
+      <c r="H67" s="8"/>
+      <c r="I67" s="8"/>
+      <c r="J67" s="8"/>
+      <c r="K67" s="8"/>
+      <c r="L67" s="8"/>
+      <c r="M67" s="8"/>
+      <c r="N67" s="8"/>
+      <c r="O67" s="8"/>
+      <c r="P67" s="8"/>
+      <c r="Q67" s="8"/>
+      <c r="R67" s="8"/>
+      <c r="S67" s="8"/>
+      <c r="T67" s="8"/>
     </row>
     <row r="68" spans="1:20" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A68" s="2"/>
@@ -4774,13 +4758,13 @@
         <v>0</v>
       </c>
       <c r="Q69" s="5">
+        <v>0</v>
+      </c>
+      <c r="R69" s="5">
+        <v>0</v>
+      </c>
+      <c r="S69" s="5">
         <v>-1</v>
-      </c>
-      <c r="R69" s="5">
-        <v>0</v>
-      </c>
-      <c r="S69" s="5">
-        <v>0</v>
       </c>
       <c r="T69" s="5">
         <v>0</v>
@@ -4898,27 +4882,27 @@
         <v>0</v>
       </c>
       <c r="Q71" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R71" s="5">
         <v>0</v>
       </c>
       <c r="S71" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T71" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
         <v>24</v>
       </c>
       <c r="B72" s="6">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="C72" s="6">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="D72" s="6">
         <v>0</v>
@@ -4936,7 +4920,7 @@
         <v>0</v>
       </c>
       <c r="I72" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J72" s="6">
         <v>0</v>
@@ -4972,7 +4956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A73" s="4" t="s">
         <v>25</v>
       </c>
@@ -4980,13 +4964,13 @@
         <v>0</v>
       </c>
       <c r="C73" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D73" s="5">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="E73" s="5">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="F73" s="5">
         <v>0</v>
@@ -5042,13 +5026,13 @@
         <v>0</v>
       </c>
       <c r="C74" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D74" s="6">
+        <v>1</v>
+      </c>
+      <c r="E74" s="6">
         <v>-1</v>
-      </c>
-      <c r="E74" s="6">
-        <v>0</v>
       </c>
       <c r="F74" s="6">
         <v>0</v>
@@ -5101,13 +5085,13 @@
         <v>27</v>
       </c>
       <c r="B75" s="5">
+        <v>1</v>
+      </c>
+      <c r="C75" s="5">
         <v>-1</v>
       </c>
-      <c r="C75" s="5">
-        <v>0</v>
-      </c>
       <c r="D75" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E75" s="5">
         <v>0</v>
@@ -5152,24 +5136,24 @@
         <v>0</v>
       </c>
       <c r="S75" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T75" s="5">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="76" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
         <v>28</v>
       </c>
       <c r="B76" s="6">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="C76" s="6">
         <v>0</v>
       </c>
       <c r="D76" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E76" s="6">
         <v>0</v>
@@ -5178,7 +5162,7 @@
         <v>-1</v>
       </c>
       <c r="G76" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H76" s="6">
         <v>0</v>
@@ -5208,7 +5192,7 @@
         <v>0</v>
       </c>
       <c r="Q76" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R76" s="6">
         <v>0</v>
@@ -5220,7 +5204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:20" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A77" s="4" t="s">
         <v>29</v>
       </c>
@@ -5237,13 +5221,13 @@
         <v>0</v>
       </c>
       <c r="F77" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G77" s="5">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="H77" s="5">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I77" s="5">
         <v>0</v>
@@ -5282,7 +5266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
         <v>30</v>
       </c>
@@ -5299,13 +5283,13 @@
         <v>0</v>
       </c>
       <c r="F78" s="6">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G78" s="6">
         <v>0</v>
       </c>
       <c r="H78" s="6">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="I78" s="6">
         <v>0</v>
@@ -5338,13 +5322,13 @@
         <v>0</v>
       </c>
       <c r="S78" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T78" s="6">
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
         <v>31</v>
       </c>
@@ -5364,17 +5348,17 @@
         <v>0</v>
       </c>
       <c r="G79" s="5">
+        <v>0</v>
+      </c>
+      <c r="H79" s="5">
+        <v>0</v>
+      </c>
+      <c r="I79" s="5">
+        <v>1</v>
+      </c>
+      <c r="J79" s="5">
         <v>-1</v>
       </c>
-      <c r="H79" s="5">
-        <v>0</v>
-      </c>
-      <c r="I79" s="5">
-        <v>0</v>
-      </c>
-      <c r="J79" s="5">
-        <v>0</v>
-      </c>
       <c r="K79" s="5">
         <v>0</v>
       </c>
@@ -5397,7 +5381,7 @@
         <v>0</v>
       </c>
       <c r="R79" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S79" s="5">
         <v>0</v>
@@ -5406,7 +5390,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
         <v>32</v>
       </c>
@@ -5429,13 +5413,13 @@
         <v>0</v>
       </c>
       <c r="H80" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I80" s="6">
         <v>0</v>
       </c>
       <c r="J80" s="6">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="K80" s="6">
         <v>0</v>
@@ -5459,7 +5443,7 @@
         <v>0</v>
       </c>
       <c r="R80" s="6">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="S80" s="6">
         <v>0</v>
@@ -5468,7 +5452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
         <v>33</v>
       </c>
@@ -5494,7 +5478,7 @@
         <v>0</v>
       </c>
       <c r="I81" s="5">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="J81" s="5">
         <v>0</v>
@@ -5503,7 +5487,7 @@
         <v>0</v>
       </c>
       <c r="L81" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M81" s="5">
         <v>0</v>
@@ -5518,7 +5502,7 @@
         <v>0</v>
       </c>
       <c r="Q81" s="5">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R81" s="5">
         <v>0</v>
@@ -5527,10 +5511,10 @@
         <v>0</v>
       </c>
       <c r="T81" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="82" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
         <v>34</v>
       </c>
@@ -5559,40 +5543,40 @@
         <v>0</v>
       </c>
       <c r="J82" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K82" s="6">
+        <v>0</v>
+      </c>
+      <c r="L82" s="6">
+        <v>0</v>
+      </c>
+      <c r="M82" s="6">
+        <v>0</v>
+      </c>
+      <c r="N82" s="6">
+        <v>0</v>
+      </c>
+      <c r="O82" s="6">
+        <v>0</v>
+      </c>
+      <c r="P82" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q82" s="6">
+        <v>0</v>
+      </c>
+      <c r="R82" s="6">
+        <v>0</v>
+      </c>
+      <c r="S82" s="6">
+        <v>0</v>
+      </c>
+      <c r="T82" s="6">
         <v>-1</v>
       </c>
-      <c r="L82" s="6">
-        <v>1</v>
-      </c>
-      <c r="M82" s="6">
-        <v>0</v>
-      </c>
-      <c r="N82" s="6">
-        <v>0</v>
-      </c>
-      <c r="O82" s="6">
-        <v>0</v>
-      </c>
-      <c r="P82" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q82" s="6">
-        <v>0</v>
-      </c>
-      <c r="R82" s="6">
-        <v>0</v>
-      </c>
-      <c r="S82" s="6">
-        <v>0</v>
-      </c>
-      <c r="T82" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="83" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
         <v>35</v>
       </c>
@@ -5627,34 +5611,34 @@
         <v>0</v>
       </c>
       <c r="L83" s="5">
+        <v>0</v>
+      </c>
+      <c r="M83" s="5">
+        <v>0</v>
+      </c>
+      <c r="N83" s="5">
+        <v>1</v>
+      </c>
+      <c r="O83" s="5">
+        <v>0</v>
+      </c>
+      <c r="P83" s="5">
+        <v>0</v>
+      </c>
+      <c r="Q83" s="5">
+        <v>0</v>
+      </c>
+      <c r="R83" s="5">
+        <v>0</v>
+      </c>
+      <c r="S83" s="5">
         <v>-1</v>
       </c>
-      <c r="M83" s="5">
-        <v>0</v>
-      </c>
-      <c r="N83" s="5">
-        <v>0</v>
-      </c>
-      <c r="O83" s="5">
-        <v>0</v>
-      </c>
-      <c r="P83" s="5">
-        <v>0</v>
-      </c>
-      <c r="Q83" s="5">
-        <v>1</v>
-      </c>
-      <c r="R83" s="5">
-        <v>0</v>
-      </c>
-      <c r="S83" s="5">
-        <v>0</v>
-      </c>
       <c r="T83" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A84" s="4" t="s">
         <v>36</v>
       </c>
@@ -5680,22 +5664,22 @@
         <v>0</v>
       </c>
       <c r="I84" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J84" s="6">
+        <v>0</v>
+      </c>
+      <c r="K84" s="6">
+        <v>0</v>
+      </c>
+      <c r="L84" s="6">
+        <v>0</v>
+      </c>
+      <c r="M84" s="6">
         <v>-1</v>
       </c>
-      <c r="K84" s="6">
-        <v>0</v>
-      </c>
-      <c r="L84" s="6">
-        <v>0</v>
-      </c>
-      <c r="M84" s="6">
-        <v>0</v>
-      </c>
       <c r="N84" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O84" s="6">
         <v>0</v>
@@ -5716,7 +5700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A85" s="4" t="s">
         <v>37</v>
       </c>
@@ -5736,29 +5720,29 @@
         <v>0</v>
       </c>
       <c r="G85" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H85" s="5">
         <v>0</v>
       </c>
       <c r="I85" s="5">
+        <v>0</v>
+      </c>
+      <c r="J85" s="5">
+        <v>0</v>
+      </c>
+      <c r="K85" s="5">
+        <v>0</v>
+      </c>
+      <c r="L85" s="5">
+        <v>0</v>
+      </c>
+      <c r="M85" s="5">
+        <v>0</v>
+      </c>
+      <c r="N85" s="5">
         <v>-1</v>
       </c>
-      <c r="J85" s="5">
-        <v>0</v>
-      </c>
-      <c r="K85" s="5">
-        <v>0</v>
-      </c>
-      <c r="L85" s="5">
-        <v>0</v>
-      </c>
-      <c r="M85" s="5">
-        <v>0</v>
-      </c>
-      <c r="N85" s="5">
-        <v>0</v>
-      </c>
       <c r="O85" s="5">
         <v>0</v>
       </c>
@@ -5772,13 +5756,13 @@
         <v>0</v>
       </c>
       <c r="S85" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T85" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A86" s="4" t="s">
         <v>38</v>
       </c>
@@ -5804,16 +5788,16 @@
         <v>0</v>
       </c>
       <c r="I86" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J86" s="6">
         <v>0</v>
       </c>
       <c r="K86" s="6">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="L86" s="6">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="M86" s="6">
         <v>0</v>
@@ -5840,7 +5824,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A87" s="4" t="s">
         <v>39</v>
       </c>
@@ -5869,16 +5853,16 @@
         <v>0</v>
       </c>
       <c r="J87" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K87" s="5">
+        <v>0</v>
+      </c>
+      <c r="L87" s="5">
+        <v>1</v>
+      </c>
+      <c r="M87" s="5">
         <v>-1</v>
-      </c>
-      <c r="L87" s="5">
-        <v>0</v>
-      </c>
-      <c r="M87" s="5">
-        <v>0</v>
       </c>
       <c r="N87" s="5">
         <v>0</v>
@@ -5928,22 +5912,22 @@
         <v>0</v>
       </c>
       <c r="I88" s="6">
+        <v>0</v>
+      </c>
+      <c r="J88" s="6">
+        <v>0</v>
+      </c>
+      <c r="K88" s="6">
+        <v>0</v>
+      </c>
+      <c r="L88" s="6">
+        <v>0</v>
+      </c>
+      <c r="M88" s="6">
+        <v>1</v>
+      </c>
+      <c r="N88" s="6">
         <v>-1</v>
-      </c>
-      <c r="J88" s="6">
-        <v>0</v>
-      </c>
-      <c r="K88" s="6">
-        <v>1</v>
-      </c>
-      <c r="L88" s="6">
-        <v>0</v>
-      </c>
-      <c r="M88" s="6">
-        <v>0</v>
-      </c>
-      <c r="N88" s="6">
-        <v>0</v>
       </c>
       <c r="O88" s="6">
         <v>0</v>
@@ -5996,10 +5980,10 @@
         <v>0</v>
       </c>
       <c r="K89" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L89" s="5">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="M89" s="5">
         <v>0</v>
@@ -6011,10 +5995,10 @@
         <v>0</v>
       </c>
       <c r="P89" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q89" s="5">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R89" s="5">
         <v>0</v>
@@ -6026,7 +6010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A90" s="4" t="s">
         <v>42</v>
       </c>
@@ -6058,22 +6042,22 @@
         <v>0</v>
       </c>
       <c r="K90" s="6">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="L90" s="6">
         <v>0</v>
       </c>
       <c r="M90" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N90" s="6">
         <v>0</v>
       </c>
       <c r="O90" s="6">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="P90" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q90" s="6">
         <v>0</v>
@@ -6088,7 +6072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A91" s="4" t="s">
         <v>43</v>
       </c>
@@ -6135,22 +6119,22 @@
         <v>0</v>
       </c>
       <c r="P91" s="5">
+        <v>0</v>
+      </c>
+      <c r="Q91" s="5">
+        <v>0</v>
+      </c>
+      <c r="R91" s="5">
+        <v>1</v>
+      </c>
+      <c r="S91" s="5">
         <v>-1</v>
       </c>
-      <c r="Q91" s="5">
-        <v>1</v>
-      </c>
-      <c r="R91" s="5">
-        <v>0</v>
-      </c>
-      <c r="S91" s="5">
-        <v>0</v>
-      </c>
       <c r="T91" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A92" s="4" t="s">
         <v>44</v>
       </c>
@@ -6188,22 +6172,22 @@
         <v>0</v>
       </c>
       <c r="M92" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N92" s="6">
+        <v>0</v>
+      </c>
+      <c r="O92" s="6">
+        <v>0</v>
+      </c>
+      <c r="P92" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q92" s="6">
         <v>-1</v>
       </c>
-      <c r="O92" s="6">
-        <v>0</v>
-      </c>
-      <c r="P92" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q92" s="6">
-        <v>0</v>
-      </c>
       <c r="R92" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S92" s="6">
         <v>0</v>
@@ -6212,7 +6196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A93" s="4" t="s">
         <v>45</v>
       </c>
@@ -6232,7 +6216,7 @@
         <v>0</v>
       </c>
       <c r="G93" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H93" s="5">
         <v>0</v>
@@ -6250,25 +6234,25 @@
         <v>0</v>
       </c>
       <c r="M93" s="5">
+        <v>0</v>
+      </c>
+      <c r="N93" s="5">
+        <v>0</v>
+      </c>
+      <c r="O93" s="5">
+        <v>0</v>
+      </c>
+      <c r="P93" s="5">
+        <v>0</v>
+      </c>
+      <c r="Q93" s="5">
+        <v>0</v>
+      </c>
+      <c r="R93" s="5">
         <v>-1</v>
       </c>
-      <c r="N93" s="5">
-        <v>0</v>
-      </c>
-      <c r="O93" s="5">
-        <v>0</v>
-      </c>
-      <c r="P93" s="5">
-        <v>0</v>
-      </c>
-      <c r="Q93" s="5">
-        <v>0</v>
-      </c>
-      <c r="R93" s="5">
-        <v>0</v>
-      </c>
       <c r="S93" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T93" s="5">
         <v>0</v>
@@ -6300,7 +6284,7 @@
         <v>0</v>
       </c>
       <c r="I94" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J94" s="6">
         <v>0</v>
@@ -6318,10 +6302,10 @@
         <v>0</v>
       </c>
       <c r="O94" s="6">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="P94" s="6">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="Q94" s="6">
         <v>0</v>
@@ -6336,7 +6320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A95" s="4" t="s">
         <v>47</v>
       </c>
@@ -6377,17 +6361,17 @@
         <v>0</v>
       </c>
       <c r="N95" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O95" s="5">
+        <v>0</v>
+      </c>
+      <c r="P95" s="5">
+        <v>1</v>
+      </c>
+      <c r="Q95" s="5">
         <v>-1</v>
       </c>
-      <c r="P95" s="5">
-        <v>0</v>
-      </c>
-      <c r="Q95" s="5">
-        <v>0</v>
-      </c>
       <c r="R95" s="5">
         <v>0</v>
       </c>
@@ -6398,7 +6382,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A96" s="4" t="s">
         <v>48</v>
       </c>
@@ -6436,23 +6420,23 @@
         <v>0</v>
       </c>
       <c r="M96" s="6">
+        <v>0</v>
+      </c>
+      <c r="N96" s="6">
+        <v>0</v>
+      </c>
+      <c r="O96" s="6">
+        <v>0</v>
+      </c>
+      <c r="P96" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q96" s="6">
+        <v>1</v>
+      </c>
+      <c r="R96" s="6">
         <v>-1</v>
       </c>
-      <c r="N96" s="6">
-        <v>0</v>
-      </c>
-      <c r="O96" s="6">
-        <v>1</v>
-      </c>
-      <c r="P96" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q96" s="6">
-        <v>0</v>
-      </c>
-      <c r="R96" s="6">
-        <v>0</v>
-      </c>
       <c r="S96" s="6">
         <v>0</v>
       </c>
@@ -6460,55 +6444,55 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A97" s="4" t="s">
         <v>49</v>
       </c>
       <c r="B97" s="5">
+        <v>0</v>
+      </c>
+      <c r="C97" s="5">
+        <v>0</v>
+      </c>
+      <c r="D97" s="5">
+        <v>0</v>
+      </c>
+      <c r="E97" s="5">
+        <v>0</v>
+      </c>
+      <c r="F97" s="5">
+        <v>0</v>
+      </c>
+      <c r="G97" s="5">
+        <v>0</v>
+      </c>
+      <c r="H97" s="5">
+        <v>0</v>
+      </c>
+      <c r="I97" s="5">
+        <v>0</v>
+      </c>
+      <c r="J97" s="5">
+        <v>0</v>
+      </c>
+      <c r="K97" s="5">
+        <v>0</v>
+      </c>
+      <c r="L97" s="5">
+        <v>0</v>
+      </c>
+      <c r="M97" s="5">
+        <v>0</v>
+      </c>
+      <c r="N97" s="5">
+        <v>0</v>
+      </c>
+      <c r="O97" s="5">
+        <v>1</v>
+      </c>
+      <c r="P97" s="5">
         <v>-1</v>
       </c>
-      <c r="C97" s="5">
-        <v>0</v>
-      </c>
-      <c r="D97" s="5">
-        <v>0</v>
-      </c>
-      <c r="E97" s="5">
-        <v>0</v>
-      </c>
-      <c r="F97" s="5">
-        <v>0</v>
-      </c>
-      <c r="G97" s="5">
-        <v>1</v>
-      </c>
-      <c r="H97" s="5">
-        <v>0</v>
-      </c>
-      <c r="I97" s="5">
-        <v>0</v>
-      </c>
-      <c r="J97" s="5">
-        <v>0</v>
-      </c>
-      <c r="K97" s="5">
-        <v>0</v>
-      </c>
-      <c r="L97" s="5">
-        <v>0</v>
-      </c>
-      <c r="M97" s="5">
-        <v>0</v>
-      </c>
-      <c r="N97" s="5">
-        <v>0</v>
-      </c>
-      <c r="O97" s="5">
-        <v>0</v>
-      </c>
-      <c r="P97" s="5">
-        <v>0</v>
-      </c>
       <c r="Q97" s="5">
         <v>0</v>
       </c>
@@ -6522,7 +6506,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:20" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A98" s="4" t="s">
         <v>50</v>
       </c>
@@ -6566,47 +6550,47 @@
         <v>0</v>
       </c>
       <c r="O98" s="6">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="P98" s="6">
         <v>0</v>
       </c>
       <c r="Q98" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R98" s="6">
         <v>0</v>
       </c>
       <c r="S98" s="6">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="T98" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="99" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A99" s="9" t="s">
+      <c r="A99" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B99" s="9"/>
-      <c r="C99" s="9"/>
-      <c r="D99" s="9"/>
-      <c r="E99" s="9"/>
-      <c r="F99" s="9"/>
-      <c r="G99" s="9"/>
-      <c r="H99" s="9"/>
-      <c r="I99" s="9"/>
-      <c r="J99" s="9"/>
-      <c r="K99" s="9"/>
-      <c r="L99" s="9"/>
-      <c r="M99" s="9"/>
-      <c r="N99" s="9"/>
-      <c r="O99" s="9"/>
-      <c r="P99" s="9"/>
-      <c r="Q99" s="9"/>
-      <c r="R99" s="9"/>
-      <c r="S99" s="9"/>
-      <c r="T99" s="9"/>
+      <c r="B99" s="8"/>
+      <c r="C99" s="8"/>
+      <c r="D99" s="8"/>
+      <c r="E99" s="8"/>
+      <c r="F99" s="8"/>
+      <c r="G99" s="8"/>
+      <c r="H99" s="8"/>
+      <c r="I99" s="8"/>
+      <c r="J99" s="8"/>
+      <c r="K99" s="8"/>
+      <c r="L99" s="8"/>
+      <c r="M99" s="8"/>
+      <c r="N99" s="8"/>
+      <c r="O99" s="8"/>
+      <c r="P99" s="8"/>
+      <c r="Q99" s="8"/>
+      <c r="R99" s="8"/>
+      <c r="S99" s="8"/>
+      <c r="T99" s="8"/>
     </row>
     <row r="100" spans="1:20" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A100" s="2"/>
@@ -6854,7 +6838,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A104" s="4" t="s">
         <v>24</v>
       </c>
@@ -6916,7 +6900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A105" s="4" t="s">
         <v>25</v>
       </c>
@@ -7102,7 +7086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A108" s="4" t="s">
         <v>28</v>
       </c>
@@ -7164,7 +7148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:20" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A109" s="4" t="s">
         <v>29</v>
       </c>
@@ -7226,7 +7210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A110" s="4" t="s">
         <v>30</v>
       </c>
@@ -7288,7 +7272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A111" s="4" t="s">
         <v>31</v>
       </c>
@@ -7350,7 +7334,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A112" s="4" t="s">
         <v>32</v>
       </c>
@@ -7412,7 +7396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A113" s="4" t="s">
         <v>33</v>
       </c>
@@ -7474,7 +7458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A114" s="4" t="s">
         <v>34</v>
       </c>
@@ -7536,7 +7520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A115" s="4" t="s">
         <v>35</v>
       </c>
@@ -7598,7 +7582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A116" s="4" t="s">
         <v>36</v>
       </c>
@@ -7660,7 +7644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A117" s="4" t="s">
         <v>37</v>
       </c>
@@ -7722,7 +7706,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A118" s="4" t="s">
         <v>38</v>
       </c>
@@ -7784,7 +7768,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A119" s="4" t="s">
         <v>39</v>
       </c>
@@ -7970,7 +7954,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A122" s="4" t="s">
         <v>42</v>
       </c>
@@ -8032,7 +8016,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A123" s="4" t="s">
         <v>43</v>
       </c>
@@ -8094,7 +8078,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A124" s="4" t="s">
         <v>44</v>
       </c>
@@ -8156,7 +8140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A125" s="4" t="s">
         <v>45</v>
       </c>
@@ -8280,7 +8264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A127" s="4" t="s">
         <v>47</v>
       </c>
@@ -8342,7 +8326,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:20" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A128" s="4" t="s">
         <v>48</v>
       </c>
@@ -8404,7 +8388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:31" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:31" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A129" s="4" t="s">
         <v>49</v>
       </c>
@@ -8466,7 +8450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:31" ht="55.2" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:31" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A130" s="4" t="s">
         <v>50</v>
       </c>
@@ -8529,39 +8513,39 @@
       </c>
     </row>
     <row r="131" spans="1:31" x14ac:dyDescent="0.3">
-      <c r="A131" s="9" t="s">
+      <c r="A131" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="B131" s="9"/>
-      <c r="C131" s="9"/>
-      <c r="D131" s="9"/>
-      <c r="E131" s="9"/>
-      <c r="F131" s="9"/>
-      <c r="G131" s="9"/>
-      <c r="H131" s="9"/>
-      <c r="I131" s="9"/>
-      <c r="J131" s="9"/>
-      <c r="K131" s="9"/>
-      <c r="L131" s="9"/>
-      <c r="M131" s="9"/>
-      <c r="N131" s="9"/>
-      <c r="O131" s="9"/>
-      <c r="P131" s="9"/>
-      <c r="Q131" s="9"/>
-      <c r="R131" s="9"/>
-      <c r="S131" s="9"/>
-      <c r="T131" s="9"/>
-      <c r="U131" s="9"/>
-      <c r="V131" s="9"/>
-      <c r="W131" s="9"/>
-      <c r="X131" s="9"/>
-      <c r="Y131" s="9"/>
-      <c r="Z131" s="9"/>
-      <c r="AA131" s="9"/>
-      <c r="AB131" s="9"/>
-      <c r="AC131" s="9"/>
-      <c r="AD131" s="9"/>
-      <c r="AE131" s="9"/>
+      <c r="B131" s="8"/>
+      <c r="C131" s="8"/>
+      <c r="D131" s="8"/>
+      <c r="E131" s="8"/>
+      <c r="F131" s="8"/>
+      <c r="G131" s="8"/>
+      <c r="H131" s="8"/>
+      <c r="I131" s="8"/>
+      <c r="J131" s="8"/>
+      <c r="K131" s="8"/>
+      <c r="L131" s="8"/>
+      <c r="M131" s="8"/>
+      <c r="N131" s="8"/>
+      <c r="O131" s="8"/>
+      <c r="P131" s="8"/>
+      <c r="Q131" s="8"/>
+      <c r="R131" s="8"/>
+      <c r="S131" s="8"/>
+      <c r="T131" s="8"/>
+      <c r="U131" s="8"/>
+      <c r="V131" s="8"/>
+      <c r="W131" s="8"/>
+      <c r="X131" s="8"/>
+      <c r="Y131" s="8"/>
+      <c r="Z131" s="8"/>
+      <c r="AA131" s="8"/>
+      <c r="AB131" s="8"/>
+      <c r="AC131" s="8"/>
+      <c r="AD131" s="8"/>
+      <c r="AE131" s="8"/>
     </row>
     <row r="132" spans="1:31" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A132" s="2"/>
@@ -8679,37 +8663,37 @@
         <v>0</v>
       </c>
       <c r="H133" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I133" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J133" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K133" s="5">
+        <v>0</v>
+      </c>
+      <c r="L133" s="5">
+        <v>0</v>
+      </c>
+      <c r="M133" s="5">
         <v>9</v>
       </c>
-      <c r="L133" s="5">
-        <v>0</v>
-      </c>
-      <c r="M133" s="5">
-        <v>0</v>
-      </c>
       <c r="N133" s="5">
         <v>0</v>
       </c>
       <c r="O133" s="5">
+        <v>0</v>
+      </c>
+      <c r="P133" s="5">
+        <v>0</v>
+      </c>
+      <c r="Q133" s="5">
         <v>2</v>
       </c>
-      <c r="P133" s="5">
-        <v>1</v>
-      </c>
-      <c r="Q133" s="5">
-        <v>0</v>
-      </c>
       <c r="R133" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S133" s="5">
         <v>0</v>
@@ -8718,22 +8702,22 @@
         <v>0</v>
       </c>
       <c r="U133" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V133" s="5">
         <v>0</v>
       </c>
       <c r="W133" s="5">
+        <v>1</v>
+      </c>
+      <c r="X133" s="5">
+        <v>0</v>
+      </c>
+      <c r="Y133" s="5">
         <v>2</v>
       </c>
-      <c r="X133" s="5">
-        <v>1</v>
-      </c>
-      <c r="Y133" s="5">
-        <v>0</v>
-      </c>
       <c r="Z133" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA133" s="5">
         <v>0</v>
@@ -8742,13 +8726,13 @@
         <v>0</v>
       </c>
       <c r="AC133" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD133" s="5">
         <v>0</v>
       </c>
       <c r="AE133" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="134" spans="1:31" x14ac:dyDescent="0.3">
@@ -8774,37 +8758,37 @@
         <v>0</v>
       </c>
       <c r="H134" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I134" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J134" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K134" s="6">
+        <v>0</v>
+      </c>
+      <c r="L134" s="6">
+        <v>1</v>
+      </c>
+      <c r="M134" s="6">
         <v>9</v>
       </c>
-      <c r="L134" s="6">
-        <v>0</v>
-      </c>
-      <c r="M134" s="6">
-        <v>0</v>
-      </c>
       <c r="N134" s="6">
         <v>0</v>
       </c>
       <c r="O134" s="6">
+        <v>0</v>
+      </c>
+      <c r="P134" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q134" s="6">
         <v>2</v>
       </c>
-      <c r="P134" s="6">
-        <v>1</v>
-      </c>
-      <c r="Q134" s="6">
-        <v>0</v>
-      </c>
       <c r="R134" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S134" s="6">
         <v>0</v>
@@ -8813,22 +8797,22 @@
         <v>0</v>
       </c>
       <c r="U134" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V134" s="6">
         <v>0</v>
       </c>
       <c r="W134" s="6">
+        <v>1</v>
+      </c>
+      <c r="X134" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y134" s="6">
         <v>2</v>
       </c>
-      <c r="X134" s="6">
-        <v>1</v>
-      </c>
-      <c r="Y134" s="6">
-        <v>0</v>
-      </c>
       <c r="Z134" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA134" s="6">
         <v>0</v>
@@ -8837,37 +8821,37 @@
         <v>0</v>
       </c>
       <c r="AC134" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD134" s="6">
         <v>0</v>
       </c>
       <c r="AE134" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="135" spans="1:31" x14ac:dyDescent="0.3">
-      <c r="A135" s="9" t="s">
+      <c r="A135" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B135" s="9"/>
-      <c r="C135" s="9"/>
-      <c r="D135" s="9"/>
-      <c r="E135" s="9"/>
-      <c r="F135" s="9"/>
-      <c r="G135" s="9"/>
-      <c r="H135" s="9"/>
-      <c r="I135" s="9"/>
-      <c r="J135" s="9"/>
-      <c r="K135" s="9"/>
-      <c r="L135" s="9"/>
-      <c r="M135" s="9"/>
-      <c r="N135" s="9"/>
-      <c r="O135" s="9"/>
-      <c r="P135" s="9"/>
-      <c r="Q135" s="9"/>
-      <c r="R135" s="9"/>
-      <c r="S135" s="9"/>
+      <c r="B135" s="8"/>
+      <c r="C135" s="8"/>
+      <c r="D135" s="8"/>
+      <c r="E135" s="8"/>
+      <c r="F135" s="8"/>
+      <c r="G135" s="8"/>
+      <c r="H135" s="8"/>
+      <c r="I135" s="8"/>
+      <c r="J135" s="8"/>
+      <c r="K135" s="8"/>
+      <c r="L135" s="8"/>
+      <c r="M135" s="8"/>
+      <c r="N135" s="8"/>
+      <c r="O135" s="8"/>
+      <c r="P135" s="8"/>
+      <c r="Q135" s="8"/>
+      <c r="R135" s="8"/>
+      <c r="S135" s="8"/>
     </row>
     <row r="136" spans="1:31" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A136" s="3" t="s">
@@ -8945,16 +8929,16 @@
         <v>58</v>
       </c>
       <c r="F137" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="G137" s="5" t="s">
         <v>58</v>
-      </c>
-      <c r="G137" s="5" t="s">
-        <v>59</v>
       </c>
       <c r="H137" s="5" t="s">
         <v>58</v>
       </c>
       <c r="I137" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J137" s="5" t="s">
         <v>58</v>
@@ -9006,10 +8990,10 @@
         <v>5</v>
       </c>
       <c r="E139" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F139" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="F139" s="3" t="s">
-        <v>7</v>
       </c>
       <c r="G139" s="3" t="s">
         <v>8</v>
@@ -9068,16 +9052,16 @@
         <v>58</v>
       </c>
       <c r="F140" t="s">
+        <v>59</v>
+      </c>
+      <c r="G140" t="s">
         <v>58</v>
-      </c>
-      <c r="G140" t="s">
-        <v>59</v>
       </c>
       <c r="H140" t="s">
         <v>58</v>
       </c>
       <c r="I140" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J140" t="s">
         <v>58</v>
@@ -9107,7 +9091,7 @@
         <v>58</v>
       </c>
       <c r="S140" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="141" spans="1:31" x14ac:dyDescent="0.3">
@@ -9129,43 +9113,43 @@
         <v>1</v>
       </c>
       <c r="E142">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F142">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G142">
         <v>1</v>
       </c>
       <c r="H142">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I142">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J142">
         <v>0</v>
       </c>
       <c r="K142">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L142">
         <v>0</v>
       </c>
       <c r="M142">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N142">
         <v>0</v>
       </c>
       <c r="O142">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P142">
         <v>0</v>
       </c>
       <c r="Q142">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R142">
         <v>0</v>
@@ -9180,62 +9164,62 @@
       </c>
     </row>
     <row r="144" spans="1:31" x14ac:dyDescent="0.3">
-      <c r="A144" s="7">
+      <c r="A144" s="9">
         <v>0.5</v>
       </c>
-      <c r="B144" s="7">
+      <c r="B144" s="9">
         <v>0.16</v>
       </c>
-      <c r="C144" s="7">
+      <c r="C144" s="9">
         <v>0.5</v>
       </c>
-      <c r="D144" s="7">
-        <v>0</v>
-      </c>
-      <c r="E144" s="7">
-        <v>0</v>
-      </c>
-      <c r="F144" s="7">
-        <v>0</v>
-      </c>
-      <c r="G144" s="7">
-        <v>0</v>
-      </c>
-      <c r="H144" s="7">
+      <c r="D144" s="9">
+        <v>0</v>
+      </c>
+      <c r="E144" s="9">
+        <v>0.2</v>
+      </c>
+      <c r="F144" s="9">
         <v>0.5</v>
       </c>
-      <c r="I144" s="7">
+      <c r="G144" s="9">
+        <v>0</v>
+      </c>
+      <c r="H144" s="9">
+        <v>0</v>
+      </c>
+      <c r="I144" s="9">
+        <v>0</v>
+      </c>
+      <c r="J144" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="K144" s="9">
         <v>0.2</v>
       </c>
-      <c r="J144" s="7">
+      <c r="L144" s="9">
         <v>0.5</v>
       </c>
-      <c r="K144" s="7">
-        <v>0</v>
-      </c>
-      <c r="L144" s="7">
+      <c r="M144" s="9">
+        <v>0</v>
+      </c>
+      <c r="N144" s="9">
         <v>0.5</v>
       </c>
-      <c r="M144" s="7">
+      <c r="O144" s="9">
         <v>0.2</v>
       </c>
-      <c r="N144" s="7">
+      <c r="P144" s="9">
         <v>0.5</v>
       </c>
-      <c r="O144" s="7">
-        <v>0</v>
-      </c>
-      <c r="P144" s="7">
+      <c r="Q144" s="9">
+        <v>0</v>
+      </c>
+      <c r="R144" s="9">
         <v>0.125</v>
       </c>
-      <c r="Q144" s="7">
+      <c r="S144" s="9">
         <v>0.33</v>
-      </c>
-      <c r="R144" s="7">
-        <v>0.2</v>
-      </c>
-      <c r="S144" s="7">
-        <v>0.5</v>
       </c>
     </row>
     <row r="145" spans="1:19" x14ac:dyDescent="0.3">
@@ -9257,43 +9241,43 @@
         <v>1</v>
       </c>
       <c r="E146">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F146">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G146">
         <v>1</v>
       </c>
       <c r="H146">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I146">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J146">
         <v>0</v>
       </c>
       <c r="K146">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L146">
         <v>0</v>
       </c>
       <c r="M146">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N146">
         <v>0</v>
       </c>
       <c r="O146">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P146">
         <v>0</v>
       </c>
       <c r="Q146">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R146">
         <v>0</v>
@@ -9321,43 +9305,43 @@
         <v>1</v>
       </c>
       <c r="E148">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F148">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G148">
         <v>1</v>
       </c>
       <c r="H148">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I148">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J148">
         <v>0</v>
       </c>
       <c r="K148">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L148">
         <v>0</v>
       </c>
       <c r="M148">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N148">
         <v>0</v>
       </c>
       <c r="O148">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P148">
         <v>0</v>
       </c>
       <c r="Q148">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R148">
         <v>0</v>
@@ -9430,24 +9414,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="R153" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="S153" s="8" t="s">
-        <v>66</v>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A135:S135"/>
     <mergeCell ref="A3:T3"/>
     <mergeCell ref="A35:T35"/>
     <mergeCell ref="A67:T67"/>
     <mergeCell ref="A99:T99"/>
     <mergeCell ref="A131:AE131"/>
+    <mergeCell ref="A135:S135"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
correzione excel, il posto "Ant_Post_Tagliatrice_Pressa_Guasta" non deve avere token
</commit_message>
<xml_diff>
--- a/Pipe_Matlab_Indici_di_Prestazione_Guasto/FOLDER/EXCEL.xlsx
+++ b/Pipe_Matlab_Indici_di_Prestazione_Guasto/FOLDER/EXCEL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lachiara\Documents\GitHub\ControlloAvanzato\Pipe_Matlab_Indici_di_Prestazione_Guasto\FOLDER\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73ACEE44-B582-4438-8923-7E9BA3F7D4E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD88F790-95DB-4DDA-8F22-F560F1867736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11520" yWindow="0" windowWidth="11520" windowHeight="12360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -442,10 +442,10 @@
     <xf numFmtId="12" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -737,28 +737,28 @@
       </c>
     </row>
     <row r="3" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
-      <c r="L3" s="8"/>
-      <c r="M3" s="8"/>
-      <c r="N3" s="8"/>
-      <c r="O3" s="8"/>
-      <c r="P3" s="8"/>
-      <c r="Q3" s="8"/>
-      <c r="R3" s="8"/>
-      <c r="S3" s="8"/>
-      <c r="T3" s="8"/>
+      <c r="A3" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="9"/>
+      <c r="O3" s="9"/>
+      <c r="P3" s="9"/>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="9"/>
+      <c r="S3" s="9"/>
+      <c r="T3" s="9"/>
     </row>
     <row r="4" spans="1:20" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
@@ -2681,28 +2681,28 @@
       </c>
     </row>
     <row r="35" spans="1:20" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="9" t="s">
+      <c r="A35" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B35" s="9"/>
-      <c r="C35" s="9"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="9"/>
-      <c r="G35" s="9"/>
-      <c r="H35" s="9"/>
-      <c r="I35" s="9"/>
-      <c r="J35" s="9"/>
-      <c r="K35" s="9"/>
-      <c r="L35" s="9"/>
-      <c r="M35" s="9"/>
-      <c r="N35" s="9"/>
-      <c r="O35" s="9"/>
-      <c r="P35" s="9"/>
-      <c r="Q35" s="9"/>
-      <c r="R35" s="9"/>
-      <c r="S35" s="9"/>
-      <c r="T35" s="9"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="8"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="8"/>
+      <c r="I35" s="8"/>
+      <c r="J35" s="8"/>
+      <c r="K35" s="8"/>
+      <c r="L35" s="8"/>
+      <c r="M35" s="8"/>
+      <c r="N35" s="8"/>
+      <c r="O35" s="8"/>
+      <c r="P35" s="8"/>
+      <c r="Q35" s="8"/>
+      <c r="R35" s="8"/>
+      <c r="S35" s="8"/>
+      <c r="T35" s="8"/>
     </row>
     <row r="36" spans="1:20" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A36" s="2"/>
@@ -4625,28 +4625,28 @@
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A67" s="9" t="s">
+      <c r="A67" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B67" s="9"/>
-      <c r="C67" s="9"/>
-      <c r="D67" s="9"/>
-      <c r="E67" s="9"/>
-      <c r="F67" s="9"/>
-      <c r="G67" s="9"/>
-      <c r="H67" s="9"/>
-      <c r="I67" s="9"/>
-      <c r="J67" s="9"/>
-      <c r="K67" s="9"/>
-      <c r="L67" s="9"/>
-      <c r="M67" s="9"/>
-      <c r="N67" s="9"/>
-      <c r="O67" s="9"/>
-      <c r="P67" s="9"/>
-      <c r="Q67" s="9"/>
-      <c r="R67" s="9"/>
-      <c r="S67" s="9"/>
-      <c r="T67" s="9"/>
+      <c r="B67" s="8"/>
+      <c r="C67" s="8"/>
+      <c r="D67" s="8"/>
+      <c r="E67" s="8"/>
+      <c r="F67" s="8"/>
+      <c r="G67" s="8"/>
+      <c r="H67" s="8"/>
+      <c r="I67" s="8"/>
+      <c r="J67" s="8"/>
+      <c r="K67" s="8"/>
+      <c r="L67" s="8"/>
+      <c r="M67" s="8"/>
+      <c r="N67" s="8"/>
+      <c r="O67" s="8"/>
+      <c r="P67" s="8"/>
+      <c r="Q67" s="8"/>
+      <c r="R67" s="8"/>
+      <c r="S67" s="8"/>
+      <c r="T67" s="8"/>
     </row>
     <row r="68" spans="1:20" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A68" s="2"/>
@@ -6569,28 +6569,28 @@
       </c>
     </row>
     <row r="99" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A99" s="9" t="s">
+      <c r="A99" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B99" s="9"/>
-      <c r="C99" s="9"/>
-      <c r="D99" s="9"/>
-      <c r="E99" s="9"/>
-      <c r="F99" s="9"/>
-      <c r="G99" s="9"/>
-      <c r="H99" s="9"/>
-      <c r="I99" s="9"/>
-      <c r="J99" s="9"/>
-      <c r="K99" s="9"/>
-      <c r="L99" s="9"/>
-      <c r="M99" s="9"/>
-      <c r="N99" s="9"/>
-      <c r="O99" s="9"/>
-      <c r="P99" s="9"/>
-      <c r="Q99" s="9"/>
-      <c r="R99" s="9"/>
-      <c r="S99" s="9"/>
-      <c r="T99" s="9"/>
+      <c r="B99" s="8"/>
+      <c r="C99" s="8"/>
+      <c r="D99" s="8"/>
+      <c r="E99" s="8"/>
+      <c r="F99" s="8"/>
+      <c r="G99" s="8"/>
+      <c r="H99" s="8"/>
+      <c r="I99" s="8"/>
+      <c r="J99" s="8"/>
+      <c r="K99" s="8"/>
+      <c r="L99" s="8"/>
+      <c r="M99" s="8"/>
+      <c r="N99" s="8"/>
+      <c r="O99" s="8"/>
+      <c r="P99" s="8"/>
+      <c r="Q99" s="8"/>
+      <c r="R99" s="8"/>
+      <c r="S99" s="8"/>
+      <c r="T99" s="8"/>
     </row>
     <row r="100" spans="1:20" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A100" s="2"/>
@@ -8513,39 +8513,39 @@
       </c>
     </row>
     <row r="131" spans="1:31" x14ac:dyDescent="0.3">
-      <c r="A131" s="9" t="s">
+      <c r="A131" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="B131" s="9"/>
-      <c r="C131" s="9"/>
-      <c r="D131" s="9"/>
-      <c r="E131" s="9"/>
-      <c r="F131" s="9"/>
-      <c r="G131" s="9"/>
-      <c r="H131" s="9"/>
-      <c r="I131" s="9"/>
-      <c r="J131" s="9"/>
-      <c r="K131" s="9"/>
-      <c r="L131" s="9"/>
-      <c r="M131" s="9"/>
-      <c r="N131" s="9"/>
-      <c r="O131" s="9"/>
-      <c r="P131" s="9"/>
-      <c r="Q131" s="9"/>
-      <c r="R131" s="9"/>
-      <c r="S131" s="9"/>
-      <c r="T131" s="9"/>
-      <c r="U131" s="9"/>
-      <c r="V131" s="9"/>
-      <c r="W131" s="9"/>
-      <c r="X131" s="9"/>
-      <c r="Y131" s="9"/>
-      <c r="Z131" s="9"/>
-      <c r="AA131" s="9"/>
-      <c r="AB131" s="9"/>
-      <c r="AC131" s="9"/>
-      <c r="AD131" s="9"/>
-      <c r="AE131" s="9"/>
+      <c r="B131" s="8"/>
+      <c r="C131" s="8"/>
+      <c r="D131" s="8"/>
+      <c r="E131" s="8"/>
+      <c r="F131" s="8"/>
+      <c r="G131" s="8"/>
+      <c r="H131" s="8"/>
+      <c r="I131" s="8"/>
+      <c r="J131" s="8"/>
+      <c r="K131" s="8"/>
+      <c r="L131" s="8"/>
+      <c r="M131" s="8"/>
+      <c r="N131" s="8"/>
+      <c r="O131" s="8"/>
+      <c r="P131" s="8"/>
+      <c r="Q131" s="8"/>
+      <c r="R131" s="8"/>
+      <c r="S131" s="8"/>
+      <c r="T131" s="8"/>
+      <c r="U131" s="8"/>
+      <c r="V131" s="8"/>
+      <c r="W131" s="8"/>
+      <c r="X131" s="8"/>
+      <c r="Y131" s="8"/>
+      <c r="Z131" s="8"/>
+      <c r="AA131" s="8"/>
+      <c r="AB131" s="8"/>
+      <c r="AC131" s="8"/>
+      <c r="AD131" s="8"/>
+      <c r="AE131" s="8"/>
     </row>
     <row r="132" spans="1:31" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A132" s="2"/>
@@ -8669,7 +8669,7 @@
         <v>1</v>
       </c>
       <c r="J133" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K133" s="5">
         <v>0</v>
@@ -8764,7 +8764,7 @@
         <v>1</v>
       </c>
       <c r="J134" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K134" s="6">
         <v>0</v>
@@ -8831,27 +8831,27 @@
       </c>
     </row>
     <row r="135" spans="1:31" x14ac:dyDescent="0.3">
-      <c r="A135" s="9" t="s">
+      <c r="A135" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B135" s="9"/>
-      <c r="C135" s="9"/>
-      <c r="D135" s="9"/>
-      <c r="E135" s="9"/>
-      <c r="F135" s="9"/>
-      <c r="G135" s="9"/>
-      <c r="H135" s="9"/>
-      <c r="I135" s="9"/>
-      <c r="J135" s="9"/>
-      <c r="K135" s="9"/>
-      <c r="L135" s="9"/>
-      <c r="M135" s="9"/>
-      <c r="N135" s="9"/>
-      <c r="O135" s="9"/>
-      <c r="P135" s="9"/>
-      <c r="Q135" s="9"/>
-      <c r="R135" s="9"/>
-      <c r="S135" s="9"/>
+      <c r="B135" s="8"/>
+      <c r="C135" s="8"/>
+      <c r="D135" s="8"/>
+      <c r="E135" s="8"/>
+      <c r="F135" s="8"/>
+      <c r="G135" s="8"/>
+      <c r="H135" s="8"/>
+      <c r="I135" s="8"/>
+      <c r="J135" s="8"/>
+      <c r="K135" s="8"/>
+      <c r="L135" s="8"/>
+      <c r="M135" s="8"/>
+      <c r="N135" s="8"/>
+      <c r="O135" s="8"/>
+      <c r="P135" s="8"/>
+      <c r="Q135" s="8"/>
+      <c r="R135" s="8"/>
+      <c r="S135" s="8"/>
     </row>
     <row r="136" spans="1:31" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A136" s="3" t="s">

</xml_diff>